<commit_message>
Coleta automática em 13-09-2026 21:57
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
@@ -7686,7 +7686,7 @@
       </c>
       <c r="P117" t="inlineStr">
         <is>
-          <t>transdermal</t>
+          <t>plus</t>
         </is>
       </c>
     </row>
@@ -7872,7 +7872,7 @@
       </c>
       <c r="P120" t="inlineStr">
         <is>
-          <t>transdermal</t>
+          <t>plus</t>
         </is>
       </c>
     </row>
@@ -7934,7 +7934,7 @@
       </c>
       <c r="P121" t="inlineStr">
         <is>
-          <t>transdermal</t>
+          <t>plus</t>
         </is>
       </c>
     </row>
@@ -9546,7 +9546,7 @@
       </c>
       <c r="P147" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>
@@ -9670,7 +9670,7 @@
       </c>
       <c r="P149" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>spoton</t>
         </is>
       </c>
     </row>
@@ -9918,7 +9918,7 @@
       </c>
       <c r="P153" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>spoton</t>
         </is>
       </c>
     </row>
@@ -9980,7 +9980,7 @@
       </c>
       <c r="P154" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>spoton</t>
         </is>
       </c>
     </row>
@@ -10042,7 +10042,7 @@
       </c>
       <c r="P155" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>
@@ -10104,7 +10104,7 @@
       </c>
       <c r="P156" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>
@@ -15622,7 +15622,7 @@
       </c>
       <c r="P245" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 15-09-2026 22:35
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
@@ -7686,7 +7686,7 @@
       </c>
       <c r="P117" t="inlineStr">
         <is>
-          <t>transdermal</t>
+          <t>plus</t>
         </is>
       </c>
     </row>
@@ -7872,7 +7872,7 @@
       </c>
       <c r="P120" t="inlineStr">
         <is>
-          <t>transdermal</t>
+          <t>plus</t>
         </is>
       </c>
     </row>
@@ -7934,7 +7934,7 @@
       </c>
       <c r="P121" t="inlineStr">
         <is>
-          <t>transdermal</t>
+          <t>plus</t>
         </is>
       </c>
     </row>
@@ -9546,7 +9546,7 @@
       </c>
       <c r="P147" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>
@@ -10042,7 +10042,7 @@
       </c>
       <c r="P155" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>
@@ -10104,7 +10104,7 @@
       </c>
       <c r="P156" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>
@@ -15622,7 +15622,7 @@
       </c>
       <c r="P245" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 17-09-2026 22:36
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
@@ -7686,7 +7686,7 @@
       </c>
       <c r="P117" t="inlineStr">
         <is>
-          <t>plus</t>
+          <t>transdermal</t>
         </is>
       </c>
     </row>
@@ -7872,7 +7872,7 @@
       </c>
       <c r="P120" t="inlineStr">
         <is>
-          <t>plus</t>
+          <t>transdermal</t>
         </is>
       </c>
     </row>
@@ -7934,7 +7934,7 @@
       </c>
       <c r="P121" t="inlineStr">
         <is>
-          <t>plus</t>
+          <t>transdermal</t>
         </is>
       </c>
     </row>
@@ -9546,7 +9546,7 @@
       </c>
       <c r="P147" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>
@@ -10042,7 +10042,7 @@
       </c>
       <c r="P155" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>
@@ -10104,7 +10104,7 @@
       </c>
       <c r="P156" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>
@@ -15622,7 +15622,7 @@
       </c>
       <c r="P245" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 18-09-2026 22:05
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
@@ -9546,7 +9546,7 @@
       </c>
       <c r="P147" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>
@@ -9670,7 +9670,7 @@
       </c>
       <c r="P149" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>spoton</t>
         </is>
       </c>
     </row>
@@ -9918,7 +9918,7 @@
       </c>
       <c r="P153" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>spoton</t>
         </is>
       </c>
     </row>
@@ -9980,7 +9980,7 @@
       </c>
       <c r="P154" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>spoton</t>
         </is>
       </c>
     </row>
@@ -10042,7 +10042,7 @@
       </c>
       <c r="P155" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>
@@ -10104,7 +10104,7 @@
       </c>
       <c r="P156" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>
@@ -15622,7 +15622,7 @@
       </c>
       <c r="P245" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 19-09-2026 21:56
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
@@ -9546,7 +9546,7 @@
       </c>
       <c r="P147" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>
@@ -10042,7 +10042,7 @@
       </c>
       <c r="P155" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>
@@ -10104,7 +10104,7 @@
       </c>
       <c r="P156" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>
@@ -15622,7 +15622,7 @@
       </c>
       <c r="P245" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 21-09-2026 22:58
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
@@ -7686,7 +7686,7 @@
       </c>
       <c r="P117" t="inlineStr">
         <is>
-          <t>transdermal</t>
+          <t>plus</t>
         </is>
       </c>
     </row>
@@ -7872,7 +7872,7 @@
       </c>
       <c r="P120" t="inlineStr">
         <is>
-          <t>transdermal</t>
+          <t>plus</t>
         </is>
       </c>
     </row>
@@ -7934,7 +7934,7 @@
       </c>
       <c r="P121" t="inlineStr">
         <is>
-          <t>transdermal</t>
+          <t>plus</t>
         </is>
       </c>
     </row>
@@ -9670,7 +9670,7 @@
       </c>
       <c r="P149" t="inlineStr">
         <is>
-          <t>spoton</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -9918,7 +9918,7 @@
       </c>
       <c r="P153" t="inlineStr">
         <is>
-          <t>spoton</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -9980,7 +9980,7 @@
       </c>
       <c r="P154" t="inlineStr">
         <is>
-          <t>spoton</t>
+          <t>spot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 25-09-2026 22:57
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
@@ -9546,7 +9546,7 @@
       </c>
       <c r="P147" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>
@@ -10042,7 +10042,7 @@
       </c>
       <c r="P155" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>
@@ -10104,7 +10104,7 @@
       </c>
       <c r="P156" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>
@@ -15622,7 +15622,7 @@
       </c>
       <c r="P245" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 26-09-2026 22:20
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
@@ -9546,7 +9546,7 @@
       </c>
       <c r="P147" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>
@@ -10042,7 +10042,7 @@
       </c>
       <c r="P155" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>
@@ -10104,7 +10104,7 @@
       </c>
       <c r="P156" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>
@@ -15622,7 +15622,7 @@
       </c>
       <c r="P245" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 29-09-2026 00:08
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
@@ -9546,7 +9546,7 @@
       </c>
       <c r="P147" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>
@@ -10042,7 +10042,7 @@
       </c>
       <c r="P155" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>
@@ -10104,7 +10104,7 @@
       </c>
       <c r="P156" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>
@@ -15622,7 +15622,7 @@
       </c>
       <c r="P245" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 29-09-2026 23:19
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
@@ -7686,7 +7686,7 @@
       </c>
       <c r="P117" t="inlineStr">
         <is>
-          <t>plus</t>
+          <t>transdermal</t>
         </is>
       </c>
     </row>
@@ -7872,7 +7872,7 @@
       </c>
       <c r="P120" t="inlineStr">
         <is>
-          <t>plus</t>
+          <t>transdermal</t>
         </is>
       </c>
     </row>
@@ -7934,7 +7934,7 @@
       </c>
       <c r="P121" t="inlineStr">
         <is>
-          <t>plus</t>
+          <t>transdermal</t>
         </is>
       </c>
     </row>
@@ -9546,7 +9546,7 @@
       </c>
       <c r="P147" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>
@@ -9670,7 +9670,7 @@
       </c>
       <c r="P149" t="inlineStr">
         <is>
-          <t>spoton</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -9918,7 +9918,7 @@
       </c>
       <c r="P153" t="inlineStr">
         <is>
-          <t>spoton</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -9980,7 +9980,7 @@
       </c>
       <c r="P154" t="inlineStr">
         <is>
-          <t>spoton</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -10042,7 +10042,7 @@
       </c>
       <c r="P155" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>
@@ -10104,7 +10104,7 @@
       </c>
       <c r="P156" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>
@@ -15622,7 +15622,7 @@
       </c>
       <c r="P245" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 01-10-2026 23:37
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
@@ -7686,7 +7686,7 @@
       </c>
       <c r="P117" t="inlineStr">
         <is>
-          <t>plus</t>
+          <t>transdermal</t>
         </is>
       </c>
     </row>
@@ -7872,7 +7872,7 @@
       </c>
       <c r="P120" t="inlineStr">
         <is>
-          <t>plus</t>
+          <t>transdermal</t>
         </is>
       </c>
     </row>
@@ -7934,7 +7934,7 @@
       </c>
       <c r="P121" t="inlineStr">
         <is>
-          <t>plus</t>
+          <t>transdermal</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 04-10-2026 22:43
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
@@ -7686,7 +7686,7 @@
       </c>
       <c r="P117" t="inlineStr">
         <is>
-          <t>plus</t>
+          <t>transdermal</t>
         </is>
       </c>
     </row>
@@ -7872,7 +7872,7 @@
       </c>
       <c r="P120" t="inlineStr">
         <is>
-          <t>plus</t>
+          <t>transdermal</t>
         </is>
       </c>
     </row>
@@ -7934,7 +7934,7 @@
       </c>
       <c r="P121" t="inlineStr">
         <is>
-          <t>plus</t>
+          <t>transdermal</t>
         </is>
       </c>
     </row>
@@ -9546,7 +9546,7 @@
       </c>
       <c r="P147" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>
@@ -10042,7 +10042,7 @@
       </c>
       <c r="P155" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>
@@ -10104,7 +10104,7 @@
       </c>
       <c r="P156" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>
@@ -15622,7 +15622,7 @@
       </c>
       <c r="P245" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 06-10-2026 01:09
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
@@ -7686,7 +7686,7 @@
       </c>
       <c r="P117" t="inlineStr">
         <is>
-          <t>transdermal</t>
+          <t>plus</t>
         </is>
       </c>
     </row>
@@ -7872,7 +7872,7 @@
       </c>
       <c r="P120" t="inlineStr">
         <is>
-          <t>transdermal</t>
+          <t>plus</t>
         </is>
       </c>
     </row>
@@ -7934,7 +7934,7 @@
       </c>
       <c r="P121" t="inlineStr">
         <is>
-          <t>transdermal</t>
+          <t>plus</t>
         </is>
       </c>
     </row>
@@ -9546,7 +9546,7 @@
       </c>
       <c r="P147" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>
@@ -10042,7 +10042,7 @@
       </c>
       <c r="P155" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>
@@ -10104,7 +10104,7 @@
       </c>
       <c r="P156" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>
@@ -15622,7 +15622,7 @@
       </c>
       <c r="P245" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 06-10-2026 23:33
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
@@ -7686,7 +7686,7 @@
       </c>
       <c r="P117" t="inlineStr">
         <is>
-          <t>plus</t>
+          <t>transdermal</t>
         </is>
       </c>
     </row>
@@ -7872,7 +7872,7 @@
       </c>
       <c r="P120" t="inlineStr">
         <is>
-          <t>plus</t>
+          <t>transdermal</t>
         </is>
       </c>
     </row>
@@ -7934,7 +7934,7 @@
       </c>
       <c r="P121" t="inlineStr">
         <is>
-          <t>plus</t>
+          <t>transdermal</t>
         </is>
       </c>
     </row>
@@ -9670,7 +9670,7 @@
       </c>
       <c r="P149" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>spoton</t>
         </is>
       </c>
     </row>
@@ -9918,7 +9918,7 @@
       </c>
       <c r="P153" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>spoton</t>
         </is>
       </c>
     </row>
@@ -9980,7 +9980,7 @@
       </c>
       <c r="P154" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>spoton</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 08-10-2026 00:02
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
@@ -9546,7 +9546,7 @@
       </c>
       <c r="P147" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>
@@ -9670,7 +9670,7 @@
       </c>
       <c r="P149" t="inlineStr">
         <is>
-          <t>spoton</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -9918,7 +9918,7 @@
       </c>
       <c r="P153" t="inlineStr">
         <is>
-          <t>spoton</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -9980,7 +9980,7 @@
       </c>
       <c r="P154" t="inlineStr">
         <is>
-          <t>spoton</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -10042,7 +10042,7 @@
       </c>
       <c r="P155" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>
@@ -10104,7 +10104,7 @@
       </c>
       <c r="P156" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>
@@ -15622,7 +15622,7 @@
       </c>
       <c r="P245" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 11-10-2026 23:22
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
@@ -7686,7 +7686,7 @@
       </c>
       <c r="P117" t="inlineStr">
         <is>
-          <t>transdermal</t>
+          <t>plus</t>
         </is>
       </c>
     </row>
@@ -7872,7 +7872,7 @@
       </c>
       <c r="P120" t="inlineStr">
         <is>
-          <t>transdermal</t>
+          <t>plus</t>
         </is>
       </c>
     </row>
@@ -7934,7 +7934,7 @@
       </c>
       <c r="P121" t="inlineStr">
         <is>
-          <t>transdermal</t>
+          <t>plus</t>
         </is>
       </c>
     </row>
@@ -9546,7 +9546,7 @@
       </c>
       <c r="P147" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>
@@ -10042,7 +10042,7 @@
       </c>
       <c r="P155" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>
@@ -10104,7 +10104,7 @@
       </c>
       <c r="P156" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>
@@ -15622,7 +15622,7 @@
       </c>
       <c r="P245" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 13-10-2026 01:47
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
@@ -9546,7 +9546,7 @@
       </c>
       <c r="P147" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>
@@ -10042,7 +10042,7 @@
       </c>
       <c r="P155" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>
@@ -10104,7 +10104,7 @@
       </c>
       <c r="P156" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>
@@ -15622,7 +15622,7 @@
       </c>
       <c r="P245" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 13-10-2026 23:42
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
@@ -7686,7 +7686,7 @@
       </c>
       <c r="P117" t="inlineStr">
         <is>
-          <t>plus</t>
+          <t>transdermal</t>
         </is>
       </c>
     </row>
@@ -7872,7 +7872,7 @@
       </c>
       <c r="P120" t="inlineStr">
         <is>
-          <t>plus</t>
+          <t>transdermal</t>
         </is>
       </c>
     </row>
@@ -7934,7 +7934,7 @@
       </c>
       <c r="P121" t="inlineStr">
         <is>
-          <t>plus</t>
+          <t>transdermal</t>
         </is>
       </c>
     </row>
@@ -9546,7 +9546,7 @@
       </c>
       <c r="P147" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>
@@ -10042,7 +10042,7 @@
       </c>
       <c r="P155" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>
@@ -10104,7 +10104,7 @@
       </c>
       <c r="P156" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>
@@ -15622,7 +15622,7 @@
       </c>
       <c r="P245" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 14-10-2026 22:56
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
@@ -7686,7 +7686,7 @@
       </c>
       <c r="P117" t="inlineStr">
         <is>
-          <t>transdermal</t>
+          <t>plus</t>
         </is>
       </c>
     </row>
@@ -7872,7 +7872,7 @@
       </c>
       <c r="P120" t="inlineStr">
         <is>
-          <t>transdermal</t>
+          <t>plus</t>
         </is>
       </c>
     </row>
@@ -7934,7 +7934,7 @@
       </c>
       <c r="P121" t="inlineStr">
         <is>
-          <t>transdermal</t>
+          <t>plus</t>
         </is>
       </c>
     </row>
@@ -9546,7 +9546,7 @@
       </c>
       <c r="P147" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>
@@ -10042,7 +10042,7 @@
       </c>
       <c r="P155" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>
@@ -10104,7 +10104,7 @@
       </c>
       <c r="P156" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>
@@ -15622,7 +15622,7 @@
       </c>
       <c r="P245" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 16-10-2026 22:21
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
@@ -7686,7 +7686,7 @@
       </c>
       <c r="P117" t="inlineStr">
         <is>
-          <t>plus</t>
+          <t>transdermal</t>
         </is>
       </c>
     </row>
@@ -7872,7 +7872,7 @@
       </c>
       <c r="P120" t="inlineStr">
         <is>
-          <t>plus</t>
+          <t>transdermal</t>
         </is>
       </c>
     </row>
@@ -7934,7 +7934,7 @@
       </c>
       <c r="P121" t="inlineStr">
         <is>
-          <t>plus</t>
+          <t>transdermal</t>
         </is>
       </c>
     </row>
@@ -9546,7 +9546,7 @@
       </c>
       <c r="P147" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>
@@ -10042,7 +10042,7 @@
       </c>
       <c r="P155" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>
@@ -10104,7 +10104,7 @@
       </c>
       <c r="P156" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>
@@ -15622,7 +15622,7 @@
       </c>
       <c r="P245" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 20-10-2026 22:51
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
@@ -7686,7 +7686,7 @@
       </c>
       <c r="P117" t="inlineStr">
         <is>
-          <t>plus</t>
+          <t>transdermal</t>
         </is>
       </c>
     </row>
@@ -7872,7 +7872,7 @@
       </c>
       <c r="P120" t="inlineStr">
         <is>
-          <t>plus</t>
+          <t>transdermal</t>
         </is>
       </c>
     </row>
@@ -7934,7 +7934,7 @@
       </c>
       <c r="P121" t="inlineStr">
         <is>
-          <t>plus</t>
+          <t>transdermal</t>
         </is>
       </c>
     </row>
@@ -9670,7 +9670,7 @@
       </c>
       <c r="P149" t="inlineStr">
         <is>
-          <t>spoton</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -9918,7 +9918,7 @@
       </c>
       <c r="P153" t="inlineStr">
         <is>
-          <t>spoton</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -9980,7 +9980,7 @@
       </c>
       <c r="P154" t="inlineStr">
         <is>
-          <t>spoton</t>
+          <t>spot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 24-10-2026 22:14
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
@@ -7686,7 +7686,7 @@
       </c>
       <c r="P117" t="inlineStr">
         <is>
-          <t>transdermal</t>
+          <t>plus</t>
         </is>
       </c>
     </row>
@@ -7872,7 +7872,7 @@
       </c>
       <c r="P120" t="inlineStr">
         <is>
-          <t>transdermal</t>
+          <t>plus</t>
         </is>
       </c>
     </row>
@@ -7934,7 +7934,7 @@
       </c>
       <c r="P121" t="inlineStr">
         <is>
-          <t>transdermal</t>
+          <t>plus</t>
         </is>
       </c>
     </row>
@@ -9546,7 +9546,7 @@
       </c>
       <c r="P147" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>
@@ -10042,7 +10042,7 @@
       </c>
       <c r="P155" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>
@@ -10104,7 +10104,7 @@
       </c>
       <c r="P156" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>
@@ -15622,7 +15622,7 @@
       </c>
       <c r="P245" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>

</xml_diff>